<commit_message>
Update PanelOLS Model HP & Building_Rest using floor data yearly
</commit_message>
<xml_diff>
--- a/Heat Pump/heat_pumps.xlsx
+++ b/Heat Pump/heat_pumps.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ittuberlin-my.sharepoint.com/personal/17281442811011116638102512442_msopseudo_tu-berlin_de/Documents/Dokumente/2. WiIng/4. Masterarbeit SS26/Code/Heat Pump/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="290" documentId="13_ncr:1_{43BD2D88-8073-4D43-9DAF-0EC65F0D6566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97030C29-3B57-2D4C-9E3C-B022CB69392B}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="13_ncr:1_{43BD2D88-8073-4D43-9DAF-0EC65F0D6566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C74477D1-6BEF-C846-8210-CF3D55DD148D}"/>
   <bookViews>
-    <workbookView xWindow="33820" yWindow="-2840" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33820" yWindow="-2840" windowWidth="30240" windowHeight="17300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documentation" sheetId="8" r:id="rId1"/>
@@ -1399,8 +1399,8 @@
         <v>18729410</v>
       </c>
       <c r="E4" s="4">
-        <f>SUM(C4:D4)</f>
-        <v>127639282</v>
+        <f>SUM(C4)</f>
+        <v>108909872</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1417,8 +1417,8 @@
         <v>93229643</v>
       </c>
       <c r="E5" s="4">
-        <f t="shared" ref="E5:E68" si="0">SUM(C5:D5)</f>
-        <v>378961390</v>
+        <f t="shared" ref="E5:E68" si="0">SUM(C5)</f>
+        <v>285731747</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="E6" s="4">
         <f t="shared" si="0"/>
-        <v>85268963</v>
+        <v>66932083</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v>29156255</v>
+        <v>23713301</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="E8" s="4">
         <f t="shared" si="0"/>
-        <v>17004919</v>
+        <v>7245195</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1490,7 +1490,7 @@
       </c>
       <c r="E9" s="4">
         <f t="shared" si="0"/>
-        <v>150771214</v>
+        <v>69149239</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="E10" s="4">
         <f t="shared" si="0"/>
-        <v>86408212</v>
+        <v>70528445</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1526,7 +1526,7 @@
       </c>
       <c r="E11" s="4">
         <f t="shared" si="0"/>
-        <v>11903569</v>
+        <v>9082825</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="E12" s="4">
         <f t="shared" si="0"/>
-        <v>72630161</v>
+        <v>59734692</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="E13" s="4">
         <f t="shared" si="0"/>
-        <v>997402420</v>
+        <v>563983513</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="E14" s="4">
         <f t="shared" si="0"/>
-        <v>1162662495</v>
+        <v>814782438</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1598,7 +1598,7 @@
       </c>
       <c r="E15" s="4">
         <f t="shared" si="0"/>
-        <v>89919131</v>
+        <v>46846238</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="E16" s="4">
         <f t="shared" si="0"/>
-        <v>90998860</v>
+        <v>62287371</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="E17" s="4">
         <f t="shared" si="0"/>
-        <v>37752949</v>
+        <v>35166847</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="E18" s="4">
         <f t="shared" si="0"/>
-        <v>699475285</v>
+        <v>535773501</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E19" s="4">
         <f t="shared" si="0"/>
-        <v>18577400</v>
+        <v>15401407</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1688,7 +1688,7 @@
       </c>
       <c r="E20" s="4">
         <f t="shared" si="0"/>
-        <v>28124026</v>
+        <v>22554183</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="E21" s="4">
         <f t="shared" si="0"/>
-        <v>10770824</v>
+        <v>7345977</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="E22" s="4">
         <f t="shared" si="0"/>
-        <v>6308061</v>
+        <v>5385667</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="E23" s="4">
         <f t="shared" si="0"/>
-        <v>319697583</v>
+        <v>160678284</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="E24" s="4">
         <f t="shared" si="0"/>
-        <v>286256803</v>
+        <v>165463102</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1778,7 +1778,7 @@
       </c>
       <c r="E25" s="4">
         <f t="shared" si="0"/>
-        <v>136152100</v>
+        <v>89529262</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="E26" s="4">
         <f t="shared" si="0"/>
-        <v>65305171</v>
+        <v>51423962</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E27" s="4">
         <f t="shared" si="0"/>
-        <v>50822658</v>
+        <v>38487132</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="E28" s="4">
         <f t="shared" si="0"/>
-        <v>8064983</v>
+        <v>6821921</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1850,7 +1850,7 @@
       </c>
       <c r="E29" s="4">
         <f t="shared" si="0"/>
-        <v>1025475472</v>
+        <v>498325510</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="E30" s="4">
         <f t="shared" si="0"/>
-        <v>123368769</v>
+        <v>89192174</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="E31" s="4">
         <f t="shared" si="0"/>
-        <v>175505382</v>
+        <v>127658239</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="E32" s="4">
         <f t="shared" si="0"/>
-        <v>179280291</v>
+        <v>151203956</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -1922,7 +1922,7 @@
       </c>
       <c r="E33" s="4">
         <f t="shared" si="0"/>
-        <v>93421183</v>
+        <v>72831990</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="E34" s="4">
         <f t="shared" si="0"/>
-        <v>40161976</v>
+        <v>31313889</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="E35" s="4">
         <f t="shared" si="0"/>
-        <v>31223377</v>
+        <v>29726256</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="E36" s="4">
         <f t="shared" si="0"/>
-        <v>110282225</v>
+        <v>80859025</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="E37" s="4">
         <f t="shared" si="0"/>
-        <v>84591452</v>
+        <v>62426542</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="E38" s="4">
         <f t="shared" si="0"/>
-        <v>8178748</v>
+        <v>5800745</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="E39" s="4">
         <f t="shared" si="0"/>
-        <v>120144375</v>
+        <v>95478485</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="E40" s="4">
         <f t="shared" si="0"/>
-        <v>523328214</v>
+        <v>437047547</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="E41" s="4">
         <f t="shared" si="0"/>
-        <v>2149374638</v>
+        <v>1150954237</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="E42" s="4">
         <f t="shared" si="0"/>
-        <v>135883258</v>
+        <v>130070281</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2102,7 +2102,7 @@
       </c>
       <c r="E43" s="4">
         <f t="shared" si="0"/>
-        <v>86586766</v>
+        <v>60861268</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="E44" s="4">
         <f t="shared" si="0"/>
-        <v>39561291</v>
+        <v>35505986</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="E45" s="4">
         <f t="shared" si="0"/>
-        <v>602605444</v>
+        <v>510537224</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="E46" s="4">
         <f t="shared" si="0"/>
-        <v>11520233</v>
+        <v>8523278</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="E47" s="4">
         <f t="shared" si="0"/>
-        <v>36748089</v>
+        <v>26821191</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="E48" s="4">
         <f t="shared" si="0"/>
-        <v>5997800</v>
+        <v>5252699</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="E49" s="4">
         <f t="shared" si="0"/>
-        <v>5782286</v>
+        <v>4814197</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="E50" s="4">
         <f t="shared" si="0"/>
-        <v>174446100</v>
+        <v>151102615</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="E51" s="4">
         <f t="shared" si="0"/>
-        <v>312826267</v>
+        <v>192607767</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="E52" s="4">
         <f t="shared" si="0"/>
-        <v>100131893</v>
+        <v>79667659</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="E53" s="4">
         <f t="shared" si="0"/>
-        <v>146975010</v>
+        <v>121854798</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="E54" s="4">
         <f t="shared" si="0"/>
-        <v>45322861</v>
+        <v>33380145</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="E55" s="4">
         <f t="shared" si="0"/>
-        <v>29865616</v>
+        <v>26142651</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E56" s="4">
         <f t="shared" si="0"/>
-        <v>949207038</v>
+        <v>631174030</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="E57" s="4">
         <f t="shared" si="0"/>
-        <v>137870549</v>
+        <v>77495365</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="E58" s="4">
         <f t="shared" si="0"/>
-        <v>99771613</v>
+        <v>73752394</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -2390,7 +2390,7 @@
       </c>
       <c r="E59" s="4">
         <f t="shared" si="0"/>
-        <v>91761161</v>
+        <v>84466520</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="E60" s="4">
         <f t="shared" si="0"/>
-        <v>57900793</v>
+        <v>46880469</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="E61" s="4">
         <f t="shared" si="0"/>
-        <v>41101083</v>
+        <v>33659750</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="E62" s="4">
         <f t="shared" si="0"/>
-        <v>16557492</v>
+        <v>15991437</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="E63" s="4">
         <f t="shared" si="0"/>
-        <v>88675430</v>
+        <v>78905383</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="E64" s="4">
         <f t="shared" si="0"/>
-        <v>86342707</v>
+        <v>68540851</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="E65" s="4">
         <f t="shared" si="0"/>
-        <v>4816345</v>
+        <v>2350354</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="E66" s="4">
         <f t="shared" si="0"/>
-        <v>78884739</v>
+        <v>60198395</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="E67" s="4">
         <f t="shared" si="0"/>
-        <v>539371676</v>
+        <v>481521196</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="E68" s="4">
         <f t="shared" si="0"/>
-        <v>1089198815</v>
+        <v>579776398</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -2569,8 +2569,8 @@
         <v>1949244</v>
       </c>
       <c r="E69" s="4">
-        <f t="shared" ref="E69:E132" si="1">SUM(C69:D69)</f>
-        <v>111475226</v>
+        <f t="shared" ref="E69:E132" si="1">SUM(C69)</f>
+        <v>109525982</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="E70" s="4">
         <f t="shared" si="1"/>
-        <v>47882392</v>
+        <v>37164058</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="E71" s="4">
         <f t="shared" si="1"/>
-        <v>30399496</v>
+        <v>27408615</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="E72" s="4">
         <f t="shared" si="1"/>
-        <v>587670096</v>
+        <v>521425889</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -2642,7 +2642,7 @@
       </c>
       <c r="E73" s="4">
         <f t="shared" si="1"/>
-        <v>10402157</v>
+        <v>8400767</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -2660,7 +2660,7 @@
       </c>
       <c r="E74" s="4">
         <f t="shared" si="1"/>
-        <v>28104958</v>
+        <v>18896748</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="E75" s="4">
         <f t="shared" si="1"/>
-        <v>4566697</v>
+        <v>3991531</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="E76" s="4">
         <f t="shared" si="1"/>
-        <v>3630818</v>
+        <v>3082472</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="E77" s="4">
         <f t="shared" si="1"/>
-        <v>130891990</v>
+        <v>95033024</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -2732,7 +2732,7 @@
       </c>
       <c r="E78" s="4">
         <f t="shared" si="1"/>
-        <v>180198874</v>
+        <v>133281509</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="E79" s="4">
         <f t="shared" si="1"/>
-        <v>108767838</v>
+        <v>98418792</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="E80" s="4">
         <f t="shared" si="1"/>
-        <v>62699679</v>
+        <v>54611294</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="E81" s="4">
         <f t="shared" si="1"/>
-        <v>24156448</v>
+        <v>20460551</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="E82" s="4">
         <f t="shared" si="1"/>
-        <v>12939606</v>
+        <v>7221994</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="E83" s="4">
         <f t="shared" si="1"/>
-        <v>569781205</v>
+        <v>474875721</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="E84" s="4">
         <f t="shared" si="1"/>
-        <v>96963208</v>
+        <v>76898507</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="E85" s="4">
         <f t="shared" si="1"/>
-        <v>82764367</v>
+        <v>59158946</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E86" s="4">
         <f t="shared" si="1"/>
-        <v>85146471</v>
+        <v>58861537</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="E87" s="4">
         <f t="shared" si="1"/>
-        <v>55750486</v>
+        <v>44125387</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="E88" s="4">
         <f t="shared" si="1"/>
-        <v>32455422</v>
+        <v>25724039</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="E89" s="4">
         <f t="shared" si="1"/>
-        <v>8646821</v>
+        <v>6646625</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="E90" s="4">
         <f t="shared" si="1"/>
-        <v>96759108</v>
+        <v>49552533</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="E91" s="4">
         <f t="shared" si="1"/>
-        <v>60888907</v>
+        <v>34519989</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -2984,7 +2984,7 @@
       </c>
       <c r="E92" s="4">
         <f t="shared" si="1"/>
-        <v>4599914</v>
+        <v>2091875</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="E93" s="4">
         <f t="shared" si="1"/>
-        <v>99224404</v>
+        <v>75976827</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="E94" s="4">
         <f t="shared" si="1"/>
-        <v>600147170</v>
+        <v>461473394</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="E95" s="4">
         <f t="shared" si="1"/>
-        <v>872405804</v>
+        <v>408888005</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="E96" s="4">
         <f t="shared" si="1"/>
-        <v>138645153</v>
+        <v>128156521</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="E97" s="4">
         <f t="shared" si="1"/>
-        <v>75746290</v>
+        <v>64388096</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="E98" s="4">
         <f t="shared" si="1"/>
-        <v>45688328</v>
+        <v>35846153</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="E99" s="4">
         <f t="shared" si="1"/>
-        <v>561288464</v>
+        <v>487488587</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="E100" s="4">
         <f t="shared" si="1"/>
-        <v>11207348</v>
+        <v>8908314</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="E101" s="4">
         <f t="shared" si="1"/>
-        <v>27850422</v>
+        <v>18896748</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="E102" s="4">
         <f t="shared" si="1"/>
-        <v>4557205</v>
+        <v>3328443</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="E103" s="4">
         <f t="shared" si="1"/>
-        <v>4326453</v>
+        <v>3965651</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="E104" s="4">
         <f t="shared" si="1"/>
-        <v>161269276</v>
+        <v>99091934</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="E105" s="4">
         <f t="shared" si="1"/>
-        <v>179783760</v>
+        <v>126541879</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="E106" s="4">
         <f t="shared" si="1"/>
-        <v>128688274</v>
+        <v>101377272</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="E107" s="4">
         <f t="shared" si="1"/>
-        <v>54915587</v>
+        <v>47559009</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="E108" s="4">
         <f t="shared" si="1"/>
-        <v>29909117</v>
+        <v>26371618</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="E109" s="4">
         <f t="shared" si="1"/>
-        <v>10172331</v>
+        <v>5118165</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -3308,7 +3308,7 @@
       </c>
       <c r="E110" s="4">
         <f t="shared" si="1"/>
-        <v>943593573</v>
+        <v>594548143</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="E111" s="4">
         <f t="shared" si="1"/>
-        <v>94912612</v>
+        <v>71122206</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="E112" s="4">
         <f t="shared" si="1"/>
-        <v>88421923</v>
+        <v>67845852</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -3362,7 +3362,7 @@
       </c>
       <c r="E113" s="4">
         <f t="shared" si="1"/>
-        <v>76167084</v>
+        <v>44583341</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="E114" s="4">
         <f t="shared" si="1"/>
-        <v>46490726</v>
+        <v>34422126</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="E115" s="4">
         <f t="shared" si="1"/>
-        <v>30164725</v>
+        <v>23512226</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -3416,7 +3416,7 @@
       </c>
       <c r="E116" s="4">
         <f t="shared" si="1"/>
-        <v>7182815</v>
+        <v>5671068</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="E117" s="4">
         <f t="shared" si="1"/>
-        <v>86563197</v>
+        <v>33899287</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="E118" s="4">
         <f t="shared" si="1"/>
-        <v>58261721</v>
+        <v>34350642</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="E119" s="4">
         <f t="shared" si="1"/>
-        <v>5713000</v>
+        <v>3240002</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="E120" s="4">
         <f t="shared" si="1"/>
-        <v>61440541</v>
+        <v>50216123</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="E121" s="4">
         <f t="shared" si="1"/>
-        <v>465450285</v>
+        <v>304593418</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="E122" s="4">
         <f t="shared" si="1"/>
-        <v>841528063</v>
+        <v>401435920</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="E123" s="4">
         <f t="shared" si="1"/>
-        <v>104777174</v>
+        <v>93201769</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="E124" s="4">
         <f t="shared" si="1"/>
-        <v>31948010</v>
+        <v>26216373</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="E125" s="4">
         <f t="shared" si="1"/>
-        <v>34739734</v>
+        <v>21936663</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="E126" s="4">
         <f t="shared" si="1"/>
-        <v>510753692</v>
+        <v>455037228</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -3614,7 +3614,7 @@
       </c>
       <c r="E127" s="4">
         <f t="shared" si="1"/>
-        <v>10025853</v>
+        <v>8855809</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="E128" s="4">
         <f t="shared" si="1"/>
-        <v>19731448</v>
+        <v>14700621</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="E129" s="4">
         <f t="shared" si="1"/>
-        <v>4051681</v>
+        <v>2535337</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="E130" s="4">
         <f t="shared" si="1"/>
-        <v>3623198</v>
+        <v>3324913</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -3686,7 +3686,7 @@
       </c>
       <c r="E131" s="4">
         <f t="shared" si="1"/>
-        <v>160889869</v>
+        <v>90124575</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="E132" s="4">
         <f t="shared" si="1"/>
-        <v>168061822</v>
+        <v>126246233</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -3721,8 +3721,8 @@
         <v>25902202</v>
       </c>
       <c r="E133" s="4">
-        <f t="shared" ref="E133:E192" si="2">SUM(C133:D133)</f>
-        <v>131167764</v>
+        <f t="shared" ref="E133:E192" si="2">SUM(C133)</f>
+        <v>105265562</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="E134" s="4">
         <f t="shared" si="2"/>
-        <v>49261360</v>
+        <v>42305348</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="E135" s="4">
         <f t="shared" si="2"/>
-        <v>23161543</v>
+        <v>20753931</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="E136" s="4">
         <f t="shared" si="2"/>
-        <v>9718066</v>
+        <v>4814662</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="E137" s="4">
         <f t="shared" si="2"/>
-        <v>985972440</v>
+        <v>607845080</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="E138" s="4">
         <f t="shared" si="2"/>
-        <v>81281216</v>
+        <v>60883492</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="E139" s="4">
         <f t="shared" si="2"/>
-        <v>54313640</v>
+        <v>33203628</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -3848,7 +3848,7 @@
       </c>
       <c r="E140" s="4">
         <f t="shared" si="2"/>
-        <v>80778170</v>
+        <v>43669097</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="E141" s="4">
         <f t="shared" si="2"/>
-        <v>45187100</v>
+        <v>35712309</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="E142" s="4">
         <f t="shared" si="2"/>
-        <v>35340571</v>
+        <v>28766954</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -3902,7 +3902,7 @@
       </c>
       <c r="E143" s="4">
         <f t="shared" si="2"/>
-        <v>21579342</v>
+        <v>17942552</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="E144" s="4">
         <f t="shared" si="2"/>
-        <v>86725442</v>
+        <v>44752848</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -3938,7 +3938,7 @@
       </c>
       <c r="E145" s="4">
         <f t="shared" si="2"/>
-        <v>65605299</v>
+        <v>36427367</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="E146" s="4">
         <f t="shared" si="2"/>
-        <v>5356099</v>
+        <v>3161858</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E147" s="4">
         <f t="shared" si="2"/>
-        <v>71203758</v>
+        <v>54482739</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -3992,7 +3992,7 @@
       </c>
       <c r="E148" s="4">
         <f t="shared" si="2"/>
-        <v>578687532</v>
+        <v>453957748</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="E149" s="4">
         <f t="shared" si="2"/>
-        <v>687663253</v>
+        <v>289930660</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E150" s="4">
         <f t="shared" si="2"/>
-        <v>56391643</v>
+        <v>36116094</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -4046,7 +4046,7 @@
       </c>
       <c r="E151" s="4">
         <f t="shared" si="2"/>
-        <v>49136094</v>
+        <v>34969397</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="E152" s="4">
         <f t="shared" si="2"/>
-        <v>54732934</v>
+        <v>45610371</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="E153" s="4">
         <f t="shared" si="2"/>
-        <v>521977024</v>
+        <v>447780870</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -4100,7 +4100,7 @@
       </c>
       <c r="E154" s="4">
         <f t="shared" si="2"/>
-        <v>13298392</v>
+        <v>9695886</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -4118,7 +4118,7 @@
       </c>
       <c r="E155" s="4">
         <f t="shared" si="2"/>
-        <v>20434840</v>
+        <v>15239314</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="E156" s="4">
         <f t="shared" si="2"/>
-        <v>4700153</v>
+        <v>3484463</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="E157" s="4">
         <f t="shared" si="2"/>
-        <v>2258896</v>
+        <v>1933819</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E158" s="4">
         <f t="shared" si="2"/>
-        <v>127317657</v>
+        <v>69263668</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="E159" s="4">
         <f t="shared" si="2"/>
-        <v>203577478</v>
+        <v>184899076</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="E160" s="4">
         <f t="shared" si="2"/>
-        <v>130209780</v>
+        <v>95234903</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="E161" s="4">
         <f t="shared" si="2"/>
-        <v>53207491</v>
+        <v>46028086</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="E162" s="4">
         <f t="shared" si="2"/>
-        <v>25149840</v>
+        <v>21612340</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="E163" s="4">
         <f t="shared" si="2"/>
-        <v>14919327</v>
+        <v>8567064</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="E164" s="4">
         <f t="shared" si="2"/>
-        <v>1083614119</v>
+        <v>631567593</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="E165" s="4">
         <f t="shared" si="2"/>
-        <v>76249781</v>
+        <v>58724389</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="E166" s="4">
         <f t="shared" si="2"/>
-        <v>17171583</v>
+        <v>9950940</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="E167" s="4">
         <f t="shared" si="2"/>
-        <v>30767106</v>
+        <v>25269082</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="E168" s="4">
         <f t="shared" si="2"/>
-        <v>27057324</v>
+        <v>20297295</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="E169" s="4">
         <f t="shared" si="2"/>
-        <v>18298503</v>
+        <v>16286976</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="E170" s="4">
         <f t="shared" si="2"/>
-        <v>10279271</v>
+        <v>9059846</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -4406,7 +4406,7 @@
       </c>
       <c r="E171" s="4">
         <f t="shared" si="2"/>
-        <v>40695491</v>
+        <v>30353791</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="E172" s="4">
         <f t="shared" si="2"/>
-        <v>43419261</v>
+        <v>34974729</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="E173" s="4">
         <f t="shared" si="2"/>
-        <v>3904904</v>
+        <v>1744924</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="E174" s="4">
         <f t="shared" si="2"/>
-        <v>13249956</v>
+        <v>10790673</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="E175" s="4">
         <f t="shared" si="2"/>
-        <v>424818667</v>
+        <v>384436486</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -4496,7 +4496,7 @@
       </c>
       <c r="E176" s="4">
         <f t="shared" si="2"/>
-        <v>512800262</v>
+        <v>162865676</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -4514,7 +4514,7 @@
       </c>
       <c r="E177" s="4">
         <f t="shared" si="2"/>
-        <v>32706209</v>
+        <v>30293028</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -4532,7 +4532,7 @@
       </c>
       <c r="E178" s="4">
         <f t="shared" si="2"/>
-        <v>19640170</v>
+        <v>17299751</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -4550,7 +4550,7 @@
       </c>
       <c r="E179" s="4">
         <f t="shared" si="2"/>
-        <v>21354773</v>
+        <v>15987678</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -4568,7 +4568,7 @@
       </c>
       <c r="E180" s="4">
         <f t="shared" si="2"/>
-        <v>461988306</v>
+        <v>406298263</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="E181" s="4">
         <f t="shared" si="2"/>
-        <v>6696633</v>
+        <v>3822841</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="E182" s="4">
         <f t="shared" si="2"/>
-        <v>14649745</v>
+        <v>11894768</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="E183" s="4">
         <f t="shared" si="2"/>
-        <v>3461902</v>
+        <v>2821375</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="E184" s="4">
         <f t="shared" si="2"/>
-        <v>1450426</v>
+        <v>1301282</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="E185" s="4">
         <f t="shared" si="2"/>
-        <v>49505370</v>
+        <v>41784744</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="E186" s="4">
         <f t="shared" si="2"/>
-        <v>141762835</v>
+        <v>123295250</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E187" s="4">
         <f t="shared" si="2"/>
-        <v>59445738</v>
+        <v>45109787</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -4712,7 +4712,7 @@
       </c>
       <c r="E188" s="4">
         <f t="shared" si="2"/>
-        <v>50375219</v>
+        <v>48811465</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="E189" s="4">
         <f t="shared" si="2"/>
-        <v>6551218</v>
+        <v>5020061</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="E190" s="4">
         <f t="shared" si="2"/>
-        <v>5781046</v>
+        <v>4904333</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="E191" s="4">
         <f t="shared" si="2"/>
-        <v>381556573</v>
+        <v>287460651</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="E192" s="4">
         <f t="shared" si="2"/>
-        <v>59643038</v>
+        <v>52286959</v>
       </c>
     </row>
     <row r="194" spans="1:1">
@@ -4859,35 +4859,35 @@
       </c>
       <c r="B2" s="48">
         <f>'BSO data'!E4+'BSO data'!E31+'BSO data'!E58+'BSO data'!E85+'BSO data'!E112+'BSO data'!E139+'BSO data'!E166</f>
-        <v>645587790</v>
+        <v>480479871</v>
       </c>
       <c r="C2" s="49">
         <f>'BSO data'!E4/heat_spec_distribution!B2</f>
-        <v>0.19771018593768633</v>
+        <v>0.22666895862532396</v>
       </c>
       <c r="D2" s="49">
         <f>'BSO data'!E31/heat_spec_distribution!B2</f>
-        <v>0.2718536265997224</v>
+        <v>0.26568904694032436</v>
       </c>
       <c r="E2" s="49">
         <f>'BSO data'!E58/heat_spec_distribution!B2</f>
-        <v>0.15454383516144257</v>
+        <v>0.15349736472102907</v>
       </c>
       <c r="F2" s="49">
         <f>'BSO data'!E85/heat_spec_distribution!B2</f>
-        <v>0.1282000190864824</v>
+        <v>0.12312471254388928</v>
       </c>
       <c r="G2" s="49">
         <f>'BSO data'!E112/heat_spec_distribution!B2</f>
-        <v>0.13696343761396107</v>
+        <v>0.14120435859008129</v>
       </c>
       <c r="H2" s="49">
         <f>'BSO data'!E139/heat_spec_distribution!B2</f>
-        <v>8.4130525454950131E-2</v>
+        <v>6.9105138433572383E-2</v>
       </c>
       <c r="I2" s="49">
         <f>'BSO data'!E166/heat_spec_distribution!B2</f>
-        <v>2.6598370145755081E-2</v>
+        <v>2.0710420145779635E-2</v>
       </c>
     </row>
     <row r="3" spans="1:9" s="50" customFormat="1">
@@ -4896,35 +4896,35 @@
       </c>
       <c r="B3" s="48">
         <f>'BSO data'!E5+'BSO data'!E32+'BSO data'!E59+'BSO data'!E86+'BSO data'!E113+'BSO data'!E140+'BSO data'!E167</f>
-        <v>922861673</v>
+        <v>693785280</v>
       </c>
       <c r="C3" s="49">
         <f>'BSO data'!E5/heat_spec_distribution!B3</f>
-        <v>0.41063726134393275</v>
+        <v>0.41184463729181453</v>
       </c>
       <c r="D3" s="49">
         <f>'BSO data'!E32/heat_spec_distribution!B3</f>
-        <v>0.19426561557942174</v>
+        <v>0.21794056512700874</v>
       </c>
       <c r="E3" s="49">
         <f>'BSO data'!E59/heat_spec_distribution!B3</f>
-        <v>9.9431110517036278E-2</v>
+        <v>0.12174735099597385</v>
       </c>
       <c r="F3" s="49">
         <f>'BSO data'!E86/heat_spec_distribution!B3</f>
-        <v>9.2263524958414861E-2</v>
+        <v>8.4841144222604428E-2</v>
       </c>
       <c r="G3" s="49">
         <f>'BSO data'!E113/heat_spec_distribution!B3</f>
-        <v>8.2533586807651507E-2</v>
+        <v>6.4261007382572316E-2</v>
       </c>
       <c r="H3" s="49">
         <f>'BSO data'!E140/heat_spec_distribution!B3</f>
-        <v>8.7530095098011504E-2</v>
+        <v>6.2943245206932036E-2</v>
       </c>
       <c r="I3" s="49">
         <f>'BSO data'!E167/heat_spec_distribution!B3</f>
-        <v>3.3338805695531361E-2</v>
+        <v>3.6422049773094059E-2</v>
       </c>
     </row>
     <row r="4" spans="1:9" s="54" customFormat="1">
@@ -4933,35 +4933,35 @@
       </c>
       <c r="B4" s="52">
         <f>'BSO data'!E6+'BSO data'!E33+'BSO data'!E60+'BSO data'!E87+'BSO data'!E114+'BSO data'!E141+'BSO data'!E168</f>
-        <v>411076575</v>
+        <v>321201659</v>
       </c>
       <c r="C4" s="53">
         <f>'BSO data'!E6/heat_spec_distribution!B4</f>
-        <v>0.20742841646960788</v>
+        <v>0.20838025310448349</v>
       </c>
       <c r="D4" s="53">
         <f>'BSO data'!E33/heat_spec_distribution!B4</f>
-        <v>0.22725980676471288</v>
+        <v>0.22674848637690256</v>
       </c>
       <c r="E4" s="53">
         <f>'BSO data'!E60/heat_spec_distribution!B4</f>
-        <v>0.14085159924279314</v>
+        <v>0.14595338375883046</v>
       </c>
       <c r="F4" s="53">
         <f>'BSO data'!E87/heat_spec_distribution!B4</f>
-        <v>0.13562068332402546</v>
+        <v>0.13737596230784099</v>
       </c>
       <c r="G4" s="53">
         <f>'BSO data'!E114/heat_spec_distribution!B4</f>
-        <v>0.11309505047812564</v>
+        <v>0.10716671298388282</v>
       </c>
       <c r="H4" s="53">
         <f>'BSO data'!E141/heat_spec_distribution!B4</f>
-        <v>0.10992380190965637</v>
+        <v>0.11118345126604716</v>
       </c>
       <c r="I4" s="53">
         <f>'BSO data'!E168/heat_spec_distribution!B4</f>
-        <v>6.5820641811078634E-2</v>
+        <v>6.3191750202012495E-2</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="54" customFormat="1">
@@ -4970,35 +4970,35 @@
       </c>
       <c r="B5" s="52">
         <f>'BSO data'!E7+'BSO data'!E34+'BSO data'!E61+'BSO data'!E88+'BSO data'!E115+'BSO data'!E142+'BSO data'!E169</f>
-        <v>226678535</v>
+        <v>182977135</v>
       </c>
       <c r="C5" s="53">
         <f>'BSO data'!E7/heat_spec_distribution!B5</f>
-        <v>0.12862380198460344</v>
+        <v>0.12959707233365525</v>
       </c>
       <c r="D5" s="53">
         <f>'BSO data'!E34/heat_spec_distribution!B5</f>
-        <v>0.17717591125247037</v>
+        <v>0.17113553013058161</v>
       </c>
       <c r="E5" s="53">
         <f>'BSO data'!E61/heat_spec_distribution!B5</f>
-        <v>0.18131881344654005</v>
+        <v>0.18395604456261708</v>
       </c>
       <c r="F5" s="53">
         <f>'BSO data'!E88/heat_spec_distribution!B5</f>
-        <v>0.1431781884420596</v>
+        <v>0.14058608470397135</v>
       </c>
       <c r="G5" s="53">
         <f>'BSO data'!E115/heat_spec_distribution!B5</f>
-        <v>0.13307270139186314</v>
+        <v>0.12849816453842716</v>
       </c>
       <c r="H5" s="53">
         <f>'BSO data'!E142/heat_spec_distribution!B5</f>
-        <v>0.15590612053320355</v>
+        <v>0.15721611336848179</v>
       </c>
       <c r="I5" s="53">
         <f>'BSO data'!E169/heat_spec_distribution!B5</f>
-        <v>8.0724462949259834E-2</v>
+        <v>8.9010990362265757E-2</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -5007,35 +5007,35 @@
       </c>
       <c r="B6" s="31">
         <f>'BSO data'!E8+'BSO data'!E35+'BSO data'!E62+'BSO data'!E89+'BSO data'!E116+'BSO data'!E143+'BSO data'!E170</f>
-        <v>112474037</v>
+        <v>92282979</v>
       </c>
       <c r="C6" s="34">
         <f>'BSO data'!E8/heat_spec_distribution!B6</f>
-        <v>0.1511897274568352</v>
+        <v>7.8510631955216792E-2</v>
       </c>
       <c r="D6" s="34">
         <f>'BSO data'!E35/heat_spec_distribution!B6</f>
-        <v>0.27760519523274513</v>
+        <v>0.32212068056450582</v>
       </c>
       <c r="E6" s="34">
         <f>'BSO data'!E62/heat_spec_distribution!B6</f>
-        <v>0.14721168050543076</v>
+        <v>0.17328696118490064</v>
       </c>
       <c r="F6" s="34">
         <f>'BSO data'!E89/heat_spec_distribution!B6</f>
-        <v>7.6878373272935868E-2</v>
+        <v>7.2024387075757493E-2</v>
       </c>
       <c r="G6" s="34">
         <f>'BSO data'!E116/heat_spec_distribution!B6</f>
-        <v>6.3861982654717014E-2</v>
+        <v>6.1453022664125306E-2</v>
       </c>
       <c r="H6" s="34">
         <f>'BSO data'!E143/heat_spec_distribution!B6</f>
-        <v>0.19186065136081137</v>
+        <v>0.19442970084439948</v>
       </c>
       <c r="I6" s="34">
         <f>'BSO data'!E170/heat_spec_distribution!B6</f>
-        <v>9.1392389516524605E-2</v>
+        <v>9.8174615711094454E-2</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="54" customFormat="1">
@@ -5044,35 +5044,35 @@
       </c>
       <c r="B7" s="52">
         <f>'BSO data'!E9+'BSO data'!E36+'BSO data'!E63+'BSO data'!E90+'BSO data'!E117+'BSO data'!E144+'BSO data'!E171</f>
-        <v>660472107</v>
+        <v>387472106</v>
       </c>
       <c r="C7" s="53">
         <f>'BSO data'!E9/heat_spec_distribution!B7</f>
-        <v>0.22827794300781881</v>
+        <v>0.17846249556864877</v>
       </c>
       <c r="D7" s="53">
         <f>'BSO data'!E36/heat_spec_distribution!B7</f>
-        <v>0.16697484092238887</v>
+        <v>0.20868347359177386</v>
       </c>
       <c r="E7" s="53">
         <f>'BSO data'!E63/heat_spec_distribution!B7</f>
-        <v>0.13426067363053684</v>
+        <v>0.20364145387023033</v>
       </c>
       <c r="F7" s="53">
         <f>'BSO data'!E90/heat_spec_distribution!B7</f>
-        <v>0.14649991570348025</v>
+        <v>0.12788671037909499</v>
       </c>
       <c r="G7" s="53">
         <f>'BSO data'!E117/heat_spec_distribution!B7</f>
-        <v>0.13106260822003191</v>
+        <v>8.7488328772755586E-2</v>
       </c>
       <c r="H7" s="53">
         <f>'BSO data'!E144/heat_spec_distribution!B7</f>
-        <v>0.13130825826078374</v>
+        <v>0.11549953482328867</v>
       </c>
       <c r="I7" s="53">
         <f>'BSO data'!E171/heat_spec_distribution!B7</f>
-        <v>6.1615760254959566E-2</v>
+        <v>7.8338002994207789E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="58" customFormat="1">
@@ -5081,35 +5081,35 @@
       </c>
       <c r="B8" s="56">
         <f>'BSO data'!E10+'BSO data'!E37+'BSO data'!E64+'BSO data'!E91+'BSO data'!E118+'BSO data'!E145+'BSO data'!E172</f>
-        <v>485517559</v>
+        <v>341768565</v>
       </c>
       <c r="C8" s="57">
         <f>'BSO data'!E10/heat_spec_distribution!B8</f>
-        <v>0.17797134294786648</v>
+        <v>0.20636317152222586</v>
       </c>
       <c r="D8" s="57">
         <f>'BSO data'!E37/heat_spec_distribution!B8</f>
-        <v>0.17422943914578382</v>
+        <v>0.18265735469264122</v>
       </c>
       <c r="E8" s="57">
         <f>'BSO data'!E64/heat_spec_distribution!B8</f>
-        <v>0.17783642506737846</v>
+        <v>0.2005475576725437</v>
       </c>
       <c r="F8" s="57">
         <f>'BSO data'!E91/heat_spec_distribution!B8</f>
-        <v>0.12541030879585552</v>
+        <v>0.10100399081466138</v>
       </c>
       <c r="G8" s="57">
         <f>'BSO data'!E118/heat_spec_distribution!B8</f>
-        <v>0.11999920480733839</v>
+        <v>0.10050848883659035</v>
       </c>
       <c r="H8" s="57">
         <f>'BSO data'!E145/heat_spec_distribution!B8</f>
-        <v>0.13512446210004117</v>
+        <v>0.10658489612700336</v>
       </c>
       <c r="I8" s="57">
         <f>'BSO data'!E172/heat_spec_distribution!B8</f>
-        <v>8.942881713573618E-2</v>
+        <v>0.10233454033433415</v>
       </c>
     </row>
     <row r="9" spans="1:9" s="58" customFormat="1">
@@ -5118,35 +5118,35 @@
       </c>
       <c r="B9" s="56">
         <f>'BSO data'!E11+'BSO data'!E38+'BSO data'!E65+'BSO data'!E92+'BSO data'!E119+'BSO data'!E146+'BSO data'!E173</f>
-        <v>44472579</v>
+        <v>27472583</v>
       </c>
       <c r="C9" s="57">
         <f>'BSO data'!E11/heat_spec_distribution!B9</f>
-        <v>0.26766086581126763</v>
+        <v>0.33061416176265623</v>
       </c>
       <c r="D9" s="57">
         <f>'BSO data'!E38/heat_spec_distribution!B9</f>
-        <v>0.18390541281628844</v>
+        <v>0.21114669123030769</v>
       </c>
       <c r="E9" s="57">
         <f>'BSO data'!E65/heat_spec_distribution!B9</f>
-        <v>0.10829920612429515</v>
+        <v>8.5552712680857124E-2</v>
       </c>
       <c r="F9" s="57">
         <f>'BSO data'!E92/heat_spec_distribution!B9</f>
-        <v>0.10343258932656008</v>
+        <v>7.6144096097552974E-2</v>
       </c>
       <c r="G9" s="57">
         <f>'BSO data'!E119/heat_spec_distribution!B9</f>
-        <v>0.12846118054003569</v>
+        <v>0.11793583442809145</v>
       </c>
       <c r="H9" s="57">
         <f>'BSO data'!E146/heat_spec_distribution!B9</f>
-        <v>0.12043598820747499</v>
+        <v>0.11509139857726519</v>
       </c>
       <c r="I9" s="57">
         <f>'BSO data'!E173/heat_spec_distribution!B9</f>
-        <v>8.7804757174077985E-2</v>
+        <v>6.3515105223269322E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9" s="58" customFormat="1">
@@ -5155,35 +5155,35 @@
       </c>
       <c r="B10" s="56">
         <f>'BSO data'!E12+'BSO data'!E39+'BSO data'!E66+'BSO data'!E93+'BSO data'!E120+'BSO data'!E147+'BSO data'!E174</f>
-        <v>516777934</v>
+        <v>406877934</v>
       </c>
       <c r="C10" s="57">
         <f>'BSO data'!E12/heat_spec_distribution!B10</f>
-        <v>0.1405442380982157</v>
+        <v>0.1468123164427983</v>
       </c>
       <c r="D10" s="57">
         <f>'BSO data'!E39/heat_spec_distribution!B10</f>
-        <v>0.23248743240650829</v>
+        <v>0.23466125100802346</v>
       </c>
       <c r="E10" s="57">
         <f>'BSO data'!E66/heat_spec_distribution!B10</f>
-        <v>0.15264726647558446</v>
+        <v>0.14795197765627663</v>
       </c>
       <c r="F10" s="57">
         <f>'BSO data'!E93/heat_spec_distribution!B10</f>
-        <v>0.19200588390447801</v>
+        <v>0.1867312543913969</v>
       </c>
       <c r="G10" s="57">
         <f>'BSO data'!E120/heat_spec_distribution!B10</f>
-        <v>0.11889157210029018</v>
+        <v>0.12341815272783999</v>
       </c>
       <c r="H10" s="57">
         <f>'BSO data'!E147/heat_spec_distribution!B10</f>
-        <v>0.13778405252109699</v>
+        <v>0.13390438371622287</v>
       </c>
       <c r="I10" s="57">
         <f>'BSO data'!E174/heat_spec_distribution!B10</f>
-        <v>2.5639554493826357E-2</v>
+        <v>2.6520664057441856E-2</v>
       </c>
     </row>
     <row r="11" spans="1:9" s="50" customFormat="1">
@@ -5192,35 +5192,35 @@
       </c>
       <c r="B11" s="48">
         <f>'BSO data'!E13+'BSO data'!E40+'BSO data'!E67+'BSO data'!E94+'BSO data'!E121+'BSO data'!E148+'BSO data'!E175</f>
-        <v>4129205964</v>
+        <v>3087013302</v>
       </c>
       <c r="C11" s="49">
         <f>'BSO data'!E13/heat_spec_distribution!B11</f>
-        <v>0.24154823680284698</v>
+        <v>0.18269552406353706</v>
       </c>
       <c r="D11" s="49">
         <f>'BSO data'!E40/heat_spec_distribution!B11</f>
-        <v>0.12673822002645929</v>
+        <v>0.14157617873458714</v>
       </c>
       <c r="E11" s="49">
         <f>'BSO data'!E67/heat_spec_distribution!B11</f>
-        <v>0.13062358252469095</v>
+        <v>0.15598287046189088</v>
       </c>
       <c r="F11" s="49">
         <f>'BSO data'!E94/heat_spec_distribution!B11</f>
-        <v>0.14534202828154202</v>
+        <v>0.14948863151999467</v>
       </c>
       <c r="G11" s="49">
         <f>'BSO data'!E121/heat_spec_distribution!B11</f>
-        <v>0.11272149877191255</v>
+        <v>9.8669292355384866E-2</v>
       </c>
       <c r="H11" s="49">
         <f>'BSO data'!E148/heat_spec_distribution!B11</f>
-        <v>0.14014499083969648</v>
+        <v>0.14705403041376333</v>
       </c>
       <c r="I11" s="49">
         <f>'BSO data'!E175/heat_spec_distribution!B11</f>
-        <v>0.10288144275285174</v>
+        <v>0.12453347245084206</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="50" customFormat="1">
@@ -5229,35 +5229,35 @@
       </c>
       <c r="B12" s="48">
         <f>'BSO data'!E14+'BSO data'!E41+'BSO data'!E68+'BSO data'!E95+'BSO data'!E122+'BSO data'!E149+'BSO data'!E176</f>
-        <v>7315633330</v>
+        <v>3808633334</v>
       </c>
       <c r="C12" s="49">
         <f>'BSO data'!E14/heat_spec_distribution!B12</f>
-        <v>0.15892848131577966</v>
+        <v>0.21393039616766638</v>
       </c>
       <c r="D12" s="49">
         <f>'BSO data'!E41/heat_spec_distribution!B12</f>
-        <v>0.29380568175633265</v>
+        <v>0.30219612550395225</v>
       </c>
       <c r="E12" s="49">
         <f>'BSO data'!E68/heat_spec_distribution!B12</f>
-        <v>0.14888646899967031</v>
+        <v>0.15222688748330951</v>
       </c>
       <c r="F12" s="49">
         <f>'BSO data'!E95/heat_spec_distribution!B12</f>
-        <v>0.11925225946227133</v>
+        <v>0.10735819627209092</v>
       </c>
       <c r="G12" s="49">
         <f>'BSO data'!E122/heat_spec_distribution!B12</f>
-        <v>0.11503147096630115</v>
+        <v>0.10540156659774695</v>
       </c>
       <c r="H12" s="49">
         <f>'BSO data'!E149/heat_spec_distribution!B12</f>
-        <v>9.3999141561678018E-2</v>
+        <v>7.6124592360142379E-2</v>
       </c>
       <c r="I12" s="49">
         <f>'BSO data'!E176/heat_spec_distribution!B12</f>
-        <v>7.0096495937966866E-2</v>
+        <v>4.2762235615091633E-2</v>
       </c>
     </row>
     <row r="13" spans="1:9" s="46" customFormat="1">
@@ -5266,35 +5266,35 @@
       </c>
       <c r="B13" s="44">
         <f>'BSO data'!E15+'BSO data'!E42+'BSO data'!E69+'BSO data'!E96+'BSO data'!E123+'BSO data'!E150+'BSO data'!E177</f>
-        <v>669797794</v>
+        <v>574209913</v>
       </c>
       <c r="C13" s="45">
         <f>'BSO data'!E15/heat_spec_distribution!B13</f>
-        <v>0.13424817430796138</v>
+        <v>8.1583819678849742E-2</v>
       </c>
       <c r="D13" s="45">
         <f>'BSO data'!E42/heat_spec_distribution!B13</f>
-        <v>0.20287205962341523</v>
+        <v>0.22652043800574373</v>
       </c>
       <c r="E13" s="45">
         <f>'BSO data'!E69/heat_spec_distribution!B13</f>
-        <v>0.1664311632534281</v>
+        <v>0.19074206056069951</v>
       </c>
       <c r="F13" s="45">
         <f>'BSO data'!E96/heat_spec_distribution!B13</f>
-        <v>0.20699553543169777</v>
+        <v>0.22318758018376461</v>
       </c>
       <c r="G13" s="45">
         <f>'BSO data'!E123/heat_spec_distribution!B13</f>
-        <v>0.15643105268274443</v>
+        <v>0.16231306163465695</v>
       </c>
       <c r="H13" s="45">
         <f>'BSO data'!E150/heat_spec_distribution!B13</f>
-        <v>8.4192040501106818E-2</v>
+        <v>6.2897022817507503E-2</v>
       </c>
       <c r="I13" s="45">
         <f>'BSO data'!E177/heat_spec_distribution!B13</f>
-        <v>4.8829974199646291E-2</v>
+        <v>5.2756017118777955E-2</v>
       </c>
     </row>
     <row r="14" spans="1:9" s="46" customFormat="1">
@@ -5303,35 +5303,35 @@
       </c>
       <c r="B14" s="44">
         <f>'BSO data'!E16+'BSO data'!E43+'BSO data'!E70+'BSO data'!E97+'BSO data'!E124+'BSO data'!E151+'BSO data'!E178</f>
-        <v>401938582</v>
+        <v>303186314</v>
       </c>
       <c r="C14" s="45">
         <f>'BSO data'!E16/heat_spec_distribution!B14</f>
-        <v>0.22639991300959508</v>
+        <v>0.20544255503564715</v>
       </c>
       <c r="D14" s="45">
         <f>'BSO data'!E43/heat_spec_distribution!B14</f>
-        <v>0.21542287771717322</v>
+        <v>0.20073883678007973</v>
       </c>
       <c r="E14" s="45">
         <f>'BSO data'!E70/heat_spec_distribution!B14</f>
-        <v>0.11912862846294263</v>
+        <v>0.12257828366223682</v>
       </c>
       <c r="F14" s="45">
         <f>'BSO data'!E97/heat_spec_distribution!B14</f>
-        <v>0.1884523989289488</v>
+        <v>0.21237138032556444</v>
       </c>
       <c r="G14" s="45">
         <f>'BSO data'!E124/heat_spec_distribution!B14</f>
-        <v>7.9484805467119848E-2</v>
+        <v>8.6469513264375117E-2</v>
       </c>
       <c r="H14" s="45">
         <f>'BSO data'!E151/heat_spec_distribution!B14</f>
-        <v>0.12224776669983874</v>
+        <v>0.11533962908365317</v>
       </c>
       <c r="I14" s="45">
         <f>'BSO data'!E178/heat_spec_distribution!B14</f>
-        <v>4.8863609714381688E-2</v>
+        <v>5.7059801848443593E-2</v>
       </c>
     </row>
     <row r="15" spans="1:9" s="50" customFormat="1">
@@ -5340,35 +5340,35 @@
       </c>
       <c r="B15" s="48">
         <f>'BSO data'!E17+'BSO data'!E44+'BSO data'!E71+'BSO data'!E98+'BSO data'!E125+'BSO data'!E152+'BSO data'!E179</f>
-        <v>264229505</v>
+        <v>217462313</v>
       </c>
       <c r="C15" s="49">
         <f>'BSO data'!E17/heat_spec_distribution!B15</f>
-        <v>0.14287938434430325</v>
+        <v>0.1617146737513088</v>
       </c>
       <c r="D15" s="49">
         <f>'BSO data'!E44/heat_spec_distribution!B15</f>
-        <v>0.14972321505124872</v>
+        <v>0.16327420374674301</v>
       </c>
       <c r="E15" s="49">
         <f>'BSO data'!E71/heat_spec_distribution!B15</f>
-        <v>0.11504958918194999</v>
+        <v>0.12603845982269121</v>
       </c>
       <c r="F15" s="49">
         <f>'BSO data'!E98/heat_spec_distribution!B15</f>
-        <v>0.17291153007307039</v>
+        <v>0.16483846099806729</v>
       </c>
       <c r="G15" s="49">
         <f>'BSO data'!E125/heat_spec_distribution!B15</f>
-        <v>0.13147560489128571</v>
+        <v>0.10087569978159848</v>
       </c>
       <c r="H15" s="49">
         <f>'BSO data'!E152/heat_spec_distribution!B15</f>
-        <v>0.20714164377668573</v>
+        <v>0.20973919743049915</v>
       </c>
       <c r="I15" s="49">
         <f>'BSO data'!E179/heat_spec_distribution!B15</f>
-        <v>8.0819032681456224E-2</v>
+        <v>7.3519304469092078E-2</v>
       </c>
     </row>
     <row r="16" spans="1:9" s="46" customFormat="1">
@@ -5377,35 +5377,35 @@
       </c>
       <c r="B16" s="44">
         <f>'BSO data'!E18+'BSO data'!E45+'BSO data'!E72+'BSO data'!E99+'BSO data'!E126+'BSO data'!E153+'BSO data'!E180</f>
-        <v>3945758311</v>
+        <v>3364341562</v>
       </c>
       <c r="C16" s="45">
         <f>'BSO data'!E18/heat_spec_distribution!B16</f>
-        <v>0.17727271410669024</v>
+        <v>0.15925062634885939</v>
       </c>
       <c r="D16" s="45">
         <f>'BSO data'!E45/heat_spec_distribution!B16</f>
-        <v>0.15272234042314611</v>
+        <v>0.1517495220361933</v>
       </c>
       <c r="E16" s="45">
         <f>'BSO data'!E72/heat_spec_distribution!B16</f>
-        <v>0.14893717498147088</v>
+        <v>0.15498601416974678</v>
       </c>
       <c r="F16" s="45">
         <f>'BSO data'!E99/heat_spec_distribution!B16</f>
-        <v>0.14225110099501986</v>
+        <v>0.14489866085719391</v>
       </c>
       <c r="G16" s="45">
         <f>'BSO data'!E126/heat_spec_distribution!B16</f>
-        <v>0.12944373470015103</v>
+        <v>0.13525298178389891</v>
       </c>
       <c r="H16" s="45">
         <f>'BSO data'!E153/heat_spec_distribution!B16</f>
-        <v>0.13228813902382983</v>
+        <v>0.13309613835219744</v>
       </c>
       <c r="I16" s="45">
         <f>'BSO data'!E180/heat_spec_distribution!B16</f>
-        <v>0.11708479576969204</v>
+        <v>0.12076605645191028</v>
       </c>
     </row>
     <row r="17" spans="1:9" s="58" customFormat="1">
@@ -5414,35 +5414,35 @@
       </c>
       <c r="B17" s="56">
         <f>'BSO data'!E19+'BSO data'!E46+'BSO data'!E73+'BSO data'!E100+'BSO data'!E127+'BSO data'!E154+'BSO data'!E181</f>
-        <v>81728016</v>
+        <v>63608302</v>
       </c>
       <c r="C17" s="57">
         <f>'BSO data'!E19/heat_spec_distribution!B17</f>
-        <v>0.22730761015904263</v>
+        <v>0.24212888122685622</v>
       </c>
       <c r="D17" s="57">
         <f>'BSO data'!E46/heat_spec_distribution!B17</f>
-        <v>0.14095818745924285</v>
+        <v>0.13399631387739291</v>
       </c>
       <c r="E17" s="57">
         <f>'BSO data'!E73/heat_spec_distribution!B17</f>
-        <v>0.12727773790568953</v>
+        <v>0.13207029170500417</v>
       </c>
       <c r="F17" s="57">
         <f>'BSO data'!E100/heat_spec_distribution!B17</f>
-        <v>0.13712981849455394</v>
+        <v>0.14004954887806942</v>
       </c>
       <c r="G17" s="57">
         <f>'BSO data'!E127/heat_spec_distribution!B17</f>
-        <v>0.12267339268336087</v>
+        <v>0.13922410631241186</v>
       </c>
       <c r="H17" s="57">
         <f>'BSO data'!E154/heat_spec_distribution!B17</f>
-        <v>0.16271521873233777</v>
+        <v>0.15243114019927775</v>
       </c>
       <c r="I17" s="57">
         <f>'BSO data'!E181/heat_spec_distribution!B17</f>
-        <v>8.1938034565772408E-2</v>
+        <v>6.0099717800987676E-2</v>
       </c>
     </row>
     <row r="18" spans="1:9" s="58" customFormat="1">
@@ -5451,35 +5451,35 @@
       </c>
       <c r="B18" s="56">
         <f>'BSO data'!E20+'BSO data'!E47+'BSO data'!E74+'BSO data'!E101+'BSO data'!E128+'BSO data'!E155+'BSO data'!E182</f>
-        <v>175643528</v>
+        <v>129003573</v>
       </c>
       <c r="C18" s="57">
         <f>'BSO data'!E20/heat_spec_distribution!B18</f>
-        <v>0.16011991059528252</v>
+        <v>0.17483378541771089</v>
       </c>
       <c r="D18" s="57">
         <f>'BSO data'!E47/heat_spec_distribution!B18</f>
-        <v>0.20921971574153306</v>
+        <v>0.2079104506663548</v>
       </c>
       <c r="E18" s="57">
         <f>'BSO data'!E74/heat_spec_distribution!B18</f>
-        <v>0.16001134980618245</v>
+        <v>0.14648236138389747</v>
       </c>
       <c r="F18" s="57">
         <f>'BSO data'!E101/heat_spec_distribution!B18</f>
-        <v>0.15856218738671657</v>
+        <v>0.14648236138389747</v>
       </c>
       <c r="G18" s="57">
         <f>'BSO data'!E128/heat_spec_distribution!B18</f>
-        <v>0.11233803046816504</v>
+        <v>0.11395514603304825</v>
       </c>
       <c r="H18" s="57">
         <f>'BSO data'!E155/heat_spec_distribution!B18</f>
-        <v>0.11634268699043668</v>
+        <v>0.11813094510180737</v>
       </c>
       <c r="I18" s="57">
         <f>'BSO data'!E182/heat_spec_distribution!B18</f>
-        <v>8.340611901168371E-2</v>
+        <v>9.2204950013283743E-2</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="50" customFormat="1">
@@ -5488,35 +5488,35 @@
       </c>
       <c r="B19" s="48">
         <f>'BSO data'!E21+'BSO data'!E48+'BSO data'!E75+'BSO data'!E102+'BSO data'!E129+'BSO data'!E156+'BSO data'!E183</f>
-        <v>38106262</v>
+        <v>28759825</v>
       </c>
       <c r="C19" s="49">
         <f>'BSO data'!E21/heat_spec_distribution!B19</f>
-        <v>0.28265233677341534</v>
+        <v>0.25542495477632426</v>
       </c>
       <c r="D19" s="49">
         <f>'BSO data'!E48/heat_spec_distribution!B19</f>
-        <v>0.15739670293559627</v>
+        <v>0.18264015862405283</v>
       </c>
       <c r="E19" s="49">
         <f>'BSO data'!E75/heat_spec_distribution!B19</f>
-        <v>0.11984111692718641</v>
+        <v>0.13878843143169334</v>
       </c>
       <c r="F19" s="49">
         <f>'BSO data'!E102/heat_spec_distribution!B19</f>
-        <v>0.11959202400907232</v>
+        <v>0.11573238015182638</v>
       </c>
       <c r="G19" s="49">
         <f>'BSO data'!E129/heat_spec_distribution!B19</f>
-        <v>0.10632585793904424</v>
+        <v>8.8155508595758145E-2</v>
       </c>
       <c r="H19" s="49">
         <f>'BSO data'!E156/heat_spec_distribution!B19</f>
-        <v>0.12334332346741331</v>
+        <v>0.121157308850106</v>
       </c>
       <c r="I19" s="49">
         <f>'BSO data'!E183/heat_spec_distribution!B19</f>
-        <v>9.0848637948272123E-2</v>
+        <v>9.8101257570239034E-2</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -5525,35 +5525,35 @@
       </c>
       <c r="B20" s="31">
         <f>'BSO data'!E22+'BSO data'!E49+'BSO data'!E76+'BSO data'!E103+'BSO data'!E130+'BSO data'!E157+'BSO data'!E184</f>
-        <v>27380138</v>
+        <v>23808001</v>
       </c>
       <c r="C20" s="34">
         <f>'BSO data'!E22/heat_spec_distribution!B20</f>
-        <v>0.23038821060726575</v>
+        <v>0.22621248209793002</v>
       </c>
       <c r="D20" s="34">
         <f>'BSO data'!E49/heat_spec_distribution!B20</f>
-        <v>0.21118542207493621</v>
+        <v>0.20220920689645469</v>
       </c>
       <c r="E20" s="34">
         <f>'BSO data'!E76/heat_spec_distribution!B20</f>
-        <v>0.13260773192596764</v>
+        <v>0.12947210477687732</v>
       </c>
       <c r="F20" s="34">
         <f>'BSO data'!E103/heat_spec_distribution!B20</f>
-        <v>0.15801428758321087</v>
+        <v>0.16656799535584696</v>
       </c>
       <c r="G20" s="34">
         <f>'BSO data'!E130/heat_spec_distribution!B20</f>
-        <v>0.13232942799630887</v>
+        <v>0.13965527807227496</v>
       </c>
       <c r="H20" s="34">
         <f>'BSO data'!E157/heat_spec_distribution!B20</f>
-        <v>8.2501264237601721E-2</v>
+        <v>8.122559302647879E-2</v>
       </c>
       <c r="I20" s="34">
         <f>'BSO data'!E184/heat_spec_distribution!B20</f>
-        <v>5.2973655574708935E-2</v>
+        <v>5.4657339774137274E-2</v>
       </c>
     </row>
     <row r="21" spans="1:9" s="50" customFormat="1">
@@ -5562,35 +5562,35 @@
       </c>
       <c r="B21" s="48">
         <f>'BSO data'!E23+'BSO data'!E50+'BSO data'!E77+'BSO data'!E104+'BSO data'!E131+'BSO data'!E158+'BSO data'!E185</f>
-        <v>1124017845</v>
+        <v>707078844</v>
       </c>
       <c r="C21" s="49">
         <f>'BSO data'!E23/heat_spec_distribution!B21</f>
-        <v>0.2844239390167333</v>
+        <v>0.22724238656474355</v>
       </c>
       <c r="D21" s="49">
         <f>'BSO data'!E50/heat_spec_distribution!B21</f>
-        <v>0.15519869259726921</v>
+        <v>0.21369981054050599</v>
       </c>
       <c r="E21" s="49">
         <f>'BSO data'!E77/heat_spec_distribution!B21</f>
-        <v>0.11645009959784046</v>
+        <v>0.1344023015345655</v>
       </c>
       <c r="F21" s="49">
         <f>'BSO data'!E104/heat_spec_distribution!B21</f>
-        <v>0.14347572569010236</v>
+        <v>0.14014269390302958</v>
       </c>
       <c r="G21" s="49">
         <f>'BSO data'!E131/heat_spec_distribution!B21</f>
-        <v>0.14313818033734152</v>
+        <v>0.12746043212120203</v>
       </c>
       <c r="H21" s="49">
         <f>'BSO data'!E158/heat_spec_distribution!B21</f>
-        <v>0.11327013851813002</v>
+        <v>9.7957488882244079E-2</v>
       </c>
       <c r="I21" s="49">
         <f>'BSO data'!E185/heat_spec_distribution!B21</f>
-        <v>4.4043224242583091E-2</v>
+        <v>5.9094886453709257E-2</v>
       </c>
     </row>
     <row r="22" spans="1:9" s="54" customFormat="1">
@@ -5599,35 +5599,35 @@
       </c>
       <c r="B22" s="52">
         <f>'BSO data'!E24+'BSO data'!E51+'BSO data'!E78+'BSO data'!E105+'BSO data'!E132+'BSO data'!E159+'BSO data'!E186</f>
-        <v>1472467839</v>
+        <v>1052334816</v>
       </c>
       <c r="C22" s="53">
         <f>'BSO data'!E24/heat_spec_distribution!B22</f>
-        <v>0.19440614960691172</v>
+        <v>0.15723427514157243</v>
       </c>
       <c r="D22" s="53">
         <f>'BSO data'!E51/heat_spec_distribution!B22</f>
-        <v>0.21245032231906016</v>
+        <v>0.18302897905831522</v>
       </c>
       <c r="E22" s="53">
         <f>'BSO data'!E78/heat_spec_distribution!B22</f>
-        <v>0.12237881821743476</v>
+        <v>0.12665314021122343</v>
       </c>
       <c r="F22" s="53">
         <f>'BSO data'!E105/heat_spec_distribution!B22</f>
-        <v>0.12209690102440329</v>
+        <v>0.12024868613678938</v>
       </c>
       <c r="G22" s="53">
         <f>'BSO data'!E132/heat_spec_distribution!B22</f>
-        <v>0.11413615805295697</v>
+        <v>0.11996774323201714</v>
       </c>
       <c r="H22" s="53">
         <f>'BSO data'!E159/heat_spec_distribution!B22</f>
-        <v>0.1382559758576839</v>
+        <v>0.17570365741847696</v>
       </c>
       <c r="I22" s="53">
         <f>'BSO data'!E186/heat_spec_distribution!B22</f>
-        <v>9.6275674921549176E-2</v>
+        <v>0.11716351880160544</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="46" customFormat="1">
@@ -5636,35 +5636,35 @@
       </c>
       <c r="B23" s="44">
         <f>'BSO data'!E25+'BSO data'!E52+'BSO data'!E79+'BSO data'!E106+'BSO data'!E133+'BSO data'!E160+'BSO data'!E187</f>
-        <v>794563387</v>
+        <v>614603237</v>
       </c>
       <c r="C23" s="45">
         <f>'BSO data'!E25/heat_spec_distribution!B23</f>
-        <v>0.17135461088140977</v>
+        <v>0.14567001377508201</v>
       </c>
       <c r="D23" s="45">
         <f>'BSO data'!E52/heat_spec_distribution!B23</f>
-        <v>0.12602127739369395</v>
+        <v>0.12962453531626941</v>
       </c>
       <c r="E23" s="45">
         <f>'BSO data'!E79/heat_spec_distribution!B23</f>
-        <v>0.13689007042052392</v>
+        <v>0.16013386535417809</v>
       </c>
       <c r="F23" s="45">
         <f>'BSO data'!E106/heat_spec_distribution!B23</f>
-        <v>0.16196099154012492</v>
+        <v>0.1649475074274625</v>
       </c>
       <c r="G23" s="45">
         <f>'BSO data'!E133/heat_spec_distribution!B23</f>
-        <v>0.16508156069869351</v>
+        <v>0.1712740116921968</v>
       </c>
       <c r="H23" s="45">
         <f>'BSO data'!E160/heat_spec_distribution!B23</f>
-        <v>0.16387588722358282</v>
+        <v>0.15495346797205364</v>
       </c>
       <c r="I23" s="45">
         <f>'BSO data'!E187/heat_spec_distribution!B23</f>
-        <v>7.4815601841971099E-2</v>
+        <v>7.339659846275752E-2</v>
       </c>
     </row>
     <row r="24" spans="1:9" s="54" customFormat="1">
@@ -5673,35 +5673,35 @@
       </c>
       <c r="B24" s="52">
         <f>'BSO data'!E26+'BSO data'!E53+'BSO data'!E80+'BSO data'!E107+'BSO data'!E134+'BSO data'!E161+'BSO data'!E188</f>
-        <v>482739517</v>
+        <v>412593962</v>
       </c>
       <c r="C24" s="53">
         <f>'BSO data'!E26/heat_spec_distribution!B24</f>
-        <v>0.13528035037579075</v>
+        <v>0.12463575993872639</v>
       </c>
       <c r="D24" s="53">
         <f>'BSO data'!E53/heat_spec_distribution!B24</f>
-        <v>0.30446028308057488</v>
+        <v>0.29533829678292772</v>
       </c>
       <c r="E24" s="53">
         <f>'BSO data'!E80/heat_spec_distribution!B24</f>
-        <v>0.12988304622262775</v>
+        <v>0.13236086571717692</v>
       </c>
       <c r="F24" s="53">
         <f>'BSO data'!E107/heat_spec_distribution!B24</f>
-        <v>0.11375821756063115</v>
+        <v>0.11526831068846324</v>
       </c>
       <c r="G24" s="53">
         <f>'BSO data'!E134/heat_spec_distribution!B24</f>
-        <v>0.10204542670576522</v>
+        <v>0.10253506327365983</v>
       </c>
       <c r="H24" s="53">
         <f>'BSO data'!E161/heat_spec_distribution!B24</f>
-        <v>0.11021987868459503</v>
+        <v>0.11155782740223426</v>
       </c>
       <c r="I24" s="53">
         <f>'BSO data'!E188/heat_spec_distribution!B24</f>
-        <v>0.10435279737001518</v>
+        <v>0.11830387619681162</v>
       </c>
     </row>
     <row r="25" spans="1:9" s="54" customFormat="1">
@@ -5710,35 +5710,35 @@
       </c>
       <c r="B25" s="52">
         <f>'BSO data'!E27+'BSO data'!E54+'BSO data'!E81+'BSO data'!E108+'BSO data'!E135+'BSO data'!E162+'BSO data'!E189</f>
-        <v>205073685</v>
+        <v>166085778</v>
       </c>
       <c r="C25" s="53">
         <f>'BSO data'!E27/heat_spec_distribution!B25</f>
-        <v>0.24782632642506033</v>
+        <v>0.23173044955119518</v>
       </c>
       <c r="D25" s="53">
         <f>'BSO data'!E54/heat_spec_distribution!B25</f>
-        <v>0.22100768804149593</v>
+        <v>0.20098135675409848</v>
       </c>
       <c r="E25" s="53">
         <f>'BSO data'!E81/heat_spec_distribution!B25</f>
-        <v>0.11779399194977161</v>
+        <v>0.12319267336665034</v>
       </c>
       <c r="F25" s="53">
         <f>'BSO data'!E108/heat_spec_distribution!B25</f>
-        <v>0.1458457090679382</v>
+        <v>0.15878311988880831</v>
       </c>
       <c r="G25" s="53">
         <f>'BSO data'!E135/heat_spec_distribution!B25</f>
-        <v>0.1129425406287501</v>
+        <v>0.12495910998472126</v>
       </c>
       <c r="H25" s="53">
         <f>'BSO data'!E162/heat_spec_distribution!B25</f>
-        <v>0.12263806543487039</v>
+        <v>0.13012757781102727</v>
       </c>
       <c r="I25" s="53">
         <f>'BSO data'!E189/heat_spec_distribution!B25</f>
-        <v>3.1945678452113442E-2</v>
+        <v>3.0225712643499193E-2</v>
       </c>
     </row>
     <row r="26" spans="1:9" s="46" customFormat="1">
@@ -5747,35 +5747,35 @@
       </c>
       <c r="B26" s="44">
         <f>'BSO data'!E28+'BSO data'!E55+'BSO data'!E82+'BSO data'!E109+'BSO data'!E136+'BSO data'!E163+'BSO data'!E190</f>
-        <v>91460975</v>
+        <v>63590790</v>
       </c>
       <c r="C26" s="45">
         <f>'BSO data'!E28/heat_spec_distribution!B26</f>
-        <v>8.8179499507850201E-2</v>
+        <v>0.10727844393818664</v>
       </c>
       <c r="D26" s="45">
         <f>'BSO data'!E55/heat_spec_distribution!B26</f>
-        <v>0.32653944482879171</v>
+        <v>0.41110750471884372</v>
       </c>
       <c r="E26" s="45">
         <f>'BSO data'!E82/heat_spec_distribution!B26</f>
-        <v>0.14147679925782553</v>
+        <v>0.11356981097419926</v>
       </c>
       <c r="F26" s="45">
         <f>'BSO data'!E109/heat_spec_distribution!B26</f>
-        <v>0.11122045222019555</v>
+        <v>8.0485947729223059E-2</v>
       </c>
       <c r="G26" s="45">
         <f>'BSO data'!E136/heat_spec_distribution!B26</f>
-        <v>0.10625368907339988</v>
+        <v>7.5713196832434382E-2</v>
       </c>
       <c r="H26" s="45">
         <f>'BSO data'!E163/heat_spec_distribution!B26</f>
-        <v>0.16312232621618128</v>
+        <v>0.13472177338888225</v>
       </c>
       <c r="I26" s="45">
         <f>'BSO data'!E190/heat_spec_distribution!B26</f>
-        <v>6.3207788895755818E-2</v>
+        <v>7.7123322418230694E-2</v>
       </c>
     </row>
     <row r="27" spans="1:9" s="46" customFormat="1">
@@ -5784,35 +5784,35 @@
       </c>
       <c r="B27" s="44">
         <f>'BSO data'!E29+'BSO data'!E56+'BSO data'!E83+'BSO data'!E110+'BSO data'!E137+'BSO data'!E164+'BSO data'!E191</f>
-        <v>5939200420</v>
+        <v>3725796728</v>
       </c>
       <c r="C27" s="45">
         <f>'BSO data'!E29/heat_spec_distribution!B27</f>
-        <v>0.17266221031146817</v>
+        <v>0.13375005304368823</v>
       </c>
       <c r="D27" s="45">
         <f>'BSO data'!E56/heat_spec_distribution!B27</f>
-        <v>0.15982067801645258</v>
+        <v>0.16940645882707964</v>
       </c>
       <c r="E27" s="45">
         <f>'BSO data'!E83/heat_spec_distribution!B27</f>
-        <v>9.5935675630895778E-2</v>
+        <v>0.1274561538559599</v>
       </c>
       <c r="F27" s="45">
         <f>'BSO data'!E110/heat_spec_distribution!B27</f>
-        <v>0.15887552301190064</v>
+        <v>0.15957610852247225</v>
       </c>
       <c r="G27" s="45">
         <f>'BSO data'!E137/heat_spec_distribution!B27</f>
-        <v>0.16601097290466585</v>
+        <v>0.16314499270235014</v>
       </c>
       <c r="H27" s="45">
         <f>'BSO data'!E164/heat_spec_distribution!B27</f>
-        <v>0.18245117900904242</v>
+        <v>0.1695120907304635</v>
       </c>
       <c r="I27" s="45">
         <f>'BSO data'!E191/heat_spec_distribution!B27</f>
-        <v>6.4243761115574546E-2</v>
+        <v>7.7154142317986382E-2</v>
       </c>
     </row>
     <row r="28" spans="1:9" s="58" customFormat="1">
@@ -5821,35 +5821,35 @@
       </c>
       <c r="B28" s="56">
         <f>'BSO data'!E30+'BSO data'!E57+'BSO data'!E84+'BSO data'!E111+'BSO data'!E138+'BSO data'!E165+'BSO data'!E192</f>
-        <v>670289173</v>
+        <v>486603092</v>
       </c>
       <c r="C28" s="57">
         <f>'BSO data'!E30/heat_spec_distribution!B28</f>
-        <v>0.18405305347219147</v>
+        <v>0.1832955348339628</v>
       </c>
       <c r="D28" s="57">
         <f>'BSO data'!E57/heat_spec_distribution!B28</f>
-        <v>0.20568816348761162</v>
+        <v>0.15925785568168974</v>
       </c>
       <c r="E28" s="57">
         <f>'BSO data'!E84/heat_spec_distribution!B28</f>
-        <v>0.14465877102866467</v>
+        <v>0.15803127490196878</v>
       </c>
       <c r="F28" s="57">
         <f>'BSO data'!E111/heat_spec_distribution!B28</f>
-        <v>0.14159950036967103</v>
+        <v>0.14616061255936286</v>
       </c>
       <c r="G28" s="57">
         <f>'BSO data'!E138/heat_spec_distribution!B28</f>
-        <v>0.12126291050802934</v>
+        <v>0.12511941046194586</v>
       </c>
       <c r="H28" s="57">
         <f>'BSO data'!E165/heat_spec_distribution!B28</f>
-        <v>0.11375654578863383</v>
+        <v>0.12068231781807091</v>
       </c>
       <c r="I28" s="57">
         <f>'BSO data'!E192/heat_spec_distribution!B28</f>
-        <v>8.8981055345197999E-2</v>
+        <v>0.10745299374299906</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -6088,7 +6088,7 @@
       </c>
       <c r="B2" s="60">
         <f>heat_spec_distribution!B2/1000000000*(heat_spec_distribution!C2*heat_spec_distribution!C$32+heat_spec_distribution!D2*heat_spec_distribution!D$32+heat_spec_distribution!E2*heat_spec_distribution!E$32+heat_spec_distribution!F2*heat_spec_distribution!F$32+heat_spec_distribution!G2*heat_spec_distribution!G$32+heat_spec_distribution!H2*heat_spec_distribution!H$32+heat_spec_distribution!I2*heat_spec_distribution!I$32)</f>
-        <v>95.326880524999993</v>
+        <v>72.352297874999991</v>
       </c>
     </row>
     <row r="3" spans="1:42" s="50" customFormat="1">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="B3" s="60">
         <f>heat_spec_distribution!B3/1000000000*(heat_spec_distribution!C3*heat_spec_distribution!C$32+heat_spec_distribution!D3*heat_spec_distribution!D$32+heat_spec_distribution!E3*heat_spec_distribution!E$32+heat_spec_distribution!F3*heat_spec_distribution!F$32+heat_spec_distribution!G3*heat_spec_distribution!G$32+heat_spec_distribution!H3*heat_spec_distribution!H$32+heat_spec_distribution!I3*heat_spec_distribution!I$32)</f>
-        <v>146.78723839999998</v>
+        <v>112.63168229999998</v>
       </c>
     </row>
     <row r="4" spans="1:42" s="54" customFormat="1">
@@ -6106,7 +6106,7 @@
       </c>
       <c r="B4" s="62">
         <f>heat_spec_distribution!B4/1000000000*(heat_spec_distribution!C4*heat_spec_distribution!C$32+heat_spec_distribution!D4*heat_spec_distribution!D$32+heat_spec_distribution!E4*heat_spec_distribution!E$32+heat_spec_distribution!F4*heat_spec_distribution!F$32+heat_spec_distribution!G4*heat_spec_distribution!G$32+heat_spec_distribution!H4*heat_spec_distribution!H$32+heat_spec_distribution!I4*heat_spec_distribution!I$32)</f>
-        <v>58.447400624999993</v>
+        <v>45.815259099999992</v>
       </c>
     </row>
     <row r="5" spans="1:42" s="54" customFormat="1">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="B5" s="62">
         <f>heat_spec_distribution!B5/1000000000*(heat_spec_distribution!C5*heat_spec_distribution!C$32+heat_spec_distribution!D5*heat_spec_distribution!D$32+heat_spec_distribution!E5*heat_spec_distribution!E$32+heat_spec_distribution!F5*heat_spec_distribution!F$32+heat_spec_distribution!G5*heat_spec_distribution!G$32+heat_spec_distribution!H5*heat_spec_distribution!H$32+heat_spec_distribution!I5*heat_spec_distribution!I$32)</f>
-        <v>29.663627474999995</v>
+        <v>23.810151100000002</v>
       </c>
     </row>
     <row r="6" spans="1:42">
@@ -6124,7 +6124,7 @@
       </c>
       <c r="B6" s="35">
         <f>heat_spec_distribution!B6/1000000000*(heat_spec_distribution!C6*heat_spec_distribution!C$32+heat_spec_distribution!D6*heat_spec_distribution!D$32+heat_spec_distribution!E6*heat_spec_distribution!E$32+heat_spec_distribution!F6*heat_spec_distribution!F$32+heat_spec_distribution!G6*heat_spec_distribution!G$32+heat_spec_distribution!H6*heat_spec_distribution!H$32+heat_spec_distribution!I6*heat_spec_distribution!I$32)</f>
-        <v>15.280246899999998</v>
+        <v>12.246467975</v>
       </c>
     </row>
     <row r="7" spans="1:42" s="54" customFormat="1">
@@ -6133,7 +6133,7 @@
       </c>
       <c r="B7" s="62">
         <f>heat_spec_distribution!B7/1000000000*(heat_spec_distribution!C7*heat_spec_distribution!C$32+heat_spec_distribution!D7*heat_spec_distribution!D$32+heat_spec_distribution!E7*heat_spec_distribution!E$32+heat_spec_distribution!F7*heat_spec_distribution!F$32+heat_spec_distribution!G7*heat_spec_distribution!G$32+heat_spec_distribution!H7*heat_spec_distribution!H$32+heat_spec_distribution!I7*heat_spec_distribution!I$32)</f>
-        <v>92.045337575000019</v>
+        <v>54.274133099999993</v>
       </c>
     </row>
     <row r="8" spans="1:42" s="58" customFormat="1">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="B8" s="61">
         <f>heat_spec_distribution!B8/1000000000*(heat_spec_distribution!C8*heat_spec_distribution!C$32+heat_spec_distribution!D8*heat_spec_distribution!D$32+heat_spec_distribution!E8*heat_spec_distribution!E$32+heat_spec_distribution!F8*heat_spec_distribution!F$32+heat_spec_distribution!G8*heat_spec_distribution!G$32+heat_spec_distribution!H8*heat_spec_distribution!H$32+heat_spec_distribution!I8*heat_spec_distribution!I$32)</f>
-        <v>65.565198499999994</v>
+        <v>47.542313300000011</v>
       </c>
     </row>
     <row r="9" spans="1:42" s="58" customFormat="1">
@@ -6151,7 +6151,7 @@
       </c>
       <c r="B9" s="61">
         <f>heat_spec_distribution!B9/1000000000*(heat_spec_distribution!C9*heat_spec_distribution!C$32+heat_spec_distribution!D9*heat_spec_distribution!D$32+heat_spec_distribution!E9*heat_spec_distribution!E$32+heat_spec_distribution!F9*heat_spec_distribution!F$32+heat_spec_distribution!G9*heat_spec_distribution!G$32+heat_spec_distribution!H9*heat_spec_distribution!H$32+heat_spec_distribution!I9*heat_spec_distribution!I$32)</f>
-        <v>6.2776883249999988</v>
+        <v>4.0941185999999998</v>
       </c>
     </row>
     <row r="10" spans="1:42" s="58" customFormat="1">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="B10" s="61">
         <f>heat_spec_distribution!B10/1000000000*(heat_spec_distribution!C10*heat_spec_distribution!C$32+heat_spec_distribution!D10*heat_spec_distribution!D$32+heat_spec_distribution!E10*heat_spec_distribution!E$32+heat_spec_distribution!F10*heat_spec_distribution!F$32+heat_spec_distribution!G10*heat_spec_distribution!G$32+heat_spec_distribution!H10*heat_spec_distribution!H$32+heat_spec_distribution!I10*heat_spec_distribution!I$32)</f>
-        <v>71.933892925000009</v>
+        <v>56.829887274999983</v>
       </c>
     </row>
     <row r="11" spans="1:42" s="50" customFormat="1">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="B11" s="60">
         <f>heat_spec_distribution!B11/1000000000*(heat_spec_distribution!C11*heat_spec_distribution!C$32+heat_spec_distribution!D11*heat_spec_distribution!D$32+heat_spec_distribution!E11*heat_spec_distribution!E$32+heat_spec_distribution!F11*heat_spec_distribution!F$32+heat_spec_distribution!G11*heat_spec_distribution!G$32+heat_spec_distribution!H11*heat_spec_distribution!H$32+heat_spec_distribution!I11*heat_spec_distribution!I$32)</f>
-        <v>558.17459584999995</v>
+        <v>402.92037417500001</v>
       </c>
     </row>
     <row r="12" spans="1:42" s="50" customFormat="1">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="B12" s="60">
         <f>heat_spec_distribution!B12/1000000000*(heat_spec_distribution!C12*heat_spec_distribution!C$32+heat_spec_distribution!D12*heat_spec_distribution!D$32+heat_spec_distribution!E12*heat_spec_distribution!E$32+heat_spec_distribution!F12*heat_spec_distribution!F$32+heat_spec_distribution!G12*heat_spec_distribution!G$32+heat_spec_distribution!H12*heat_spec_distribution!H$32+heat_spec_distribution!I12*heat_spec_distribution!I$32)</f>
-        <v>1042.4711717749999</v>
+        <v>572.48261469999989</v>
       </c>
     </row>
     <row r="13" spans="1:42" s="46" customFormat="1">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="B13" s="59">
         <f>heat_spec_distribution!B13/1000000000*(heat_spec_distribution!C13*heat_spec_distribution!C$32+heat_spec_distribution!D13*heat_spec_distribution!D$32+heat_spec_distribution!E13*heat_spec_distribution!E$32+heat_spec_distribution!F13*heat_spec_distribution!F$32+heat_spec_distribution!G13*heat_spec_distribution!G$32+heat_spec_distribution!H13*heat_spec_distribution!H$32+heat_spec_distribution!I13*heat_spec_distribution!I$32)</f>
-        <v>92.157725450000001</v>
+        <v>78.123544549999991</v>
       </c>
     </row>
     <row r="14" spans="1:42" s="46" customFormat="1">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="B14" s="59">
         <f>heat_spec_distribution!B14/1000000000*(heat_spec_distribution!C14*heat_spec_distribution!C$32+heat_spec_distribution!D14*heat_spec_distribution!D$32+heat_spec_distribution!E14*heat_spec_distribution!E$32+heat_spec_distribution!F14*heat_spec_distribution!F$32+heat_spec_distribution!G14*heat_spec_distribution!G$32+heat_spec_distribution!H14*heat_spec_distribution!H$32+heat_spec_distribution!I14*heat_spec_distribution!I$32)</f>
-        <v>57.865117650000002</v>
+        <v>42.840646425000003</v>
       </c>
     </row>
     <row r="15" spans="1:42" s="50" customFormat="1">
@@ -6205,7 +6205,7 @@
       </c>
       <c r="B15" s="60">
         <f>heat_spec_distribution!B15/1000000000*(heat_spec_distribution!C15*heat_spec_distribution!C$32+heat_spec_distribution!D15*heat_spec_distribution!D$32+heat_spec_distribution!E15*heat_spec_distribution!E$32+heat_spec_distribution!F15*heat_spec_distribution!F$32+heat_spec_distribution!G15*heat_spec_distribution!G$32+heat_spec_distribution!H15*heat_spec_distribution!H$32+heat_spec_distribution!I15*heat_spec_distribution!I$32)</f>
-        <v>33.391463224999995</v>
+        <v>28.252806349999997</v>
       </c>
     </row>
     <row r="16" spans="1:42" s="46" customFormat="1">
@@ -6214,7 +6214,7 @@
       </c>
       <c r="B16" s="59">
         <f>heat_spec_distribution!B16/1000000000*(heat_spec_distribution!C16*heat_spec_distribution!C$32+heat_spec_distribution!D16*heat_spec_distribution!D$32+heat_spec_distribution!E16*heat_spec_distribution!E$32+heat_spec_distribution!F16*heat_spec_distribution!F$32+heat_spec_distribution!G16*heat_spec_distribution!G$32+heat_spec_distribution!H16*heat_spec_distribution!H$32+heat_spec_distribution!I16*heat_spec_distribution!I$32)</f>
-        <v>516.98564339999996</v>
+        <v>435.05087232499989</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="58" customFormat="1">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="B17" s="61">
         <f>heat_spec_distribution!B17/1000000000*(heat_spec_distribution!C17*heat_spec_distribution!C$32+heat_spec_distribution!D17*heat_spec_distribution!D$32+heat_spec_distribution!E17*heat_spec_distribution!E$32+heat_spec_distribution!F17*heat_spec_distribution!F$32+heat_spec_distribution!G17*heat_spec_distribution!G$32+heat_spec_distribution!H17*heat_spec_distribution!H$32+heat_spec_distribution!I17*heat_spec_distribution!I$32)</f>
-        <v>11.027559174999999</v>
+        <v>8.7494237500000001</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="58" customFormat="1">
@@ -6232,7 +6232,7 @@
       </c>
       <c r="B18" s="61">
         <f>heat_spec_distribution!B18/1000000000*(heat_spec_distribution!C18*heat_spec_distribution!C$32+heat_spec_distribution!D18*heat_spec_distribution!D$32+heat_spec_distribution!E18*heat_spec_distribution!E$32+heat_spec_distribution!F18*heat_spec_distribution!F$32+heat_spec_distribution!G18*heat_spec_distribution!G$32+heat_spec_distribution!H18*heat_spec_distribution!H$32+heat_spec_distribution!I18*heat_spec_distribution!I$32)</f>
-        <v>23.991012274999999</v>
+        <v>17.608899774999998</v>
       </c>
     </row>
     <row r="19" spans="1:5" s="50" customFormat="1">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="B19" s="60">
         <f>heat_spec_distribution!B19/1000000000*(heat_spec_distribution!C19*heat_spec_distribution!C$32+heat_spec_distribution!D19*heat_spec_distribution!D$32+heat_spec_distribution!E19*heat_spec_distribution!E$32+heat_spec_distribution!F19*heat_spec_distribution!F$32+heat_spec_distribution!G19*heat_spec_distribution!G$32+heat_spec_distribution!H19*heat_spec_distribution!H$32+heat_spec_distribution!I19*heat_spec_distribution!I$32)</f>
-        <v>5.3892096499999997</v>
+        <v>4.0591399250000002</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="B20" s="35">
         <f>heat_spec_distribution!B20/1000000000*(heat_spec_distribution!C20*heat_spec_distribution!C$32+heat_spec_distribution!D20*heat_spec_distribution!D$32+heat_spec_distribution!E20*heat_spec_distribution!E$32+heat_spec_distribution!F20*heat_spec_distribution!F$32+heat_spec_distribution!G20*heat_spec_distribution!G$32+heat_spec_distribution!H20*heat_spec_distribution!H$32+heat_spec_distribution!I20*heat_spec_distribution!I$32)</f>
-        <v>3.963199874999999</v>
+        <v>3.4202868749999995</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="50" customFormat="1">
@@ -6259,7 +6259,7 @@
       </c>
       <c r="B21" s="60">
         <f>heat_spec_distribution!B21/1000000000*(heat_spec_distribution!C21*heat_spec_distribution!C$32+heat_spec_distribution!D21*heat_spec_distribution!D$32+heat_spec_distribution!E21*heat_spec_distribution!E$32+heat_spec_distribution!F21*heat_spec_distribution!F$32+heat_spec_distribution!G21*heat_spec_distribution!G$32+heat_spec_distribution!H21*heat_spec_distribution!H$32+heat_spec_distribution!I21*heat_spec_distribution!I$32)</f>
-        <v>162.37312177499996</v>
+        <v>101.51652957499999</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="54" customFormat="1">
@@ -6268,7 +6268,7 @@
       </c>
       <c r="B22" s="62">
         <f>heat_spec_distribution!B22/1000000000*(heat_spec_distribution!C22*heat_spec_distribution!C$32+heat_spec_distribution!D22*heat_spec_distribution!D$32+heat_spec_distribution!E22*heat_spec_distribution!E$32+heat_spec_distribution!F22*heat_spec_distribution!F$32+heat_spec_distribution!G22*heat_spec_distribution!G$32+heat_spec_distribution!H22*heat_spec_distribution!H$32+heat_spec_distribution!I22*heat_spec_distribution!I$32)</f>
-        <v>200.66139322499998</v>
+        <v>135.26575734999994</v>
       </c>
     </row>
     <row r="23" spans="1:5" s="46" customFormat="1">
@@ -6277,7 +6277,7 @@
       </c>
       <c r="B23" s="59">
         <f>heat_spec_distribution!B23/1000000000*(heat_spec_distribution!C23*heat_spec_distribution!C$32+heat_spec_distribution!D23*heat_spec_distribution!D$32+heat_spec_distribution!E23*heat_spec_distribution!E$32+heat_spec_distribution!F23*heat_spec_distribution!F$32+heat_spec_distribution!G23*heat_spec_distribution!G$32+heat_spec_distribution!H23*heat_spec_distribution!H$32+heat_spec_distribution!I23*heat_spec_distribution!I$32)</f>
-        <v>103.009508025</v>
+        <v>79.207333799999986</v>
       </c>
     </row>
     <row r="24" spans="1:5" s="54" customFormat="1">
@@ -6286,7 +6286,7 @@
       </c>
       <c r="B24" s="62">
         <f>heat_spec_distribution!B24/1000000000*(heat_spec_distribution!C24*heat_spec_distribution!C$32+heat_spec_distribution!D24*heat_spec_distribution!D$32+heat_spec_distribution!E24*heat_spec_distribution!E$32+heat_spec_distribution!F24*heat_spec_distribution!F$32+heat_spec_distribution!G24*heat_spec_distribution!G$32+heat_spec_distribution!H24*heat_spec_distribution!H$32+heat_spec_distribution!I24*heat_spec_distribution!I$32)</f>
-        <v>66.486519949999973</v>
+        <v>55.869166774999997</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="54" customFormat="1">
@@ -6295,7 +6295,7 @@
       </c>
       <c r="B25" s="62">
         <f>heat_spec_distribution!B25/1000000000*(heat_spec_distribution!C25*heat_spec_distribution!C$32+heat_spec_distribution!D25*heat_spec_distribution!D$32+heat_spec_distribution!E25*heat_spec_distribution!E$32+heat_spec_distribution!F25*heat_spec_distribution!F$32+heat_spec_distribution!G25*heat_spec_distribution!G$32+heat_spec_distribution!H25*heat_spec_distribution!H$32+heat_spec_distribution!I25*heat_spec_distribution!I$32)</f>
-        <v>29.988092299999998</v>
+        <v>23.851808324999993</v>
       </c>
     </row>
     <row r="26" spans="1:5" s="46" customFormat="1">
@@ -6304,7 +6304,7 @@
       </c>
       <c r="B26" s="59">
         <f>heat_spec_distribution!B26/1000000000*(heat_spec_distribution!C26*heat_spec_distribution!C$32+heat_spec_distribution!D26*heat_spec_distribution!D$32+heat_spec_distribution!E26*heat_spec_distribution!E$32+heat_spec_distribution!F26*heat_spec_distribution!F$32+heat_spec_distribution!G26*heat_spec_distribution!G$32+heat_spec_distribution!H26*heat_spec_distribution!H$32+heat_spec_distribution!I26*heat_spec_distribution!I$32)</f>
-        <v>12.4317701</v>
+        <v>9.0316304999999986</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="46" customFormat="1">
@@ -6313,7 +6313,7 @@
       </c>
       <c r="B27" s="59">
         <f>heat_spec_distribution!B27/1000000000*(heat_spec_distribution!C27*heat_spec_distribution!C$32+heat_spec_distribution!D27*heat_spec_distribution!D$32+heat_spec_distribution!E27*heat_spec_distribution!E$32+heat_spec_distribution!F27*heat_spec_distribution!F$32+heat_spec_distribution!G27*heat_spec_distribution!G$32+heat_spec_distribution!H27*heat_spec_distribution!H$32+heat_spec_distribution!I27*heat_spec_distribution!I$32)</f>
-        <v>773.56883499999992</v>
+        <v>478.1955433</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="58" customFormat="1">
@@ -6322,7 +6322,7 @@
       </c>
       <c r="B28" s="61">
         <f>heat_spec_distribution!B28/1000000000*(heat_spec_distribution!C28*heat_spec_distribution!C$32+heat_spec_distribution!D28*heat_spec_distribution!D$32+heat_spec_distribution!E28*heat_spec_distribution!E$32+heat_spec_distribution!F28*heat_spec_distribution!F$32+heat_spec_distribution!G28*heat_spec_distribution!G$32+heat_spec_distribution!H28*heat_spec_distribution!H$32+heat_spec_distribution!I28*heat_spec_distribution!I$32)</f>
-        <v>92.038664650000001</v>
+        <v>64.932201799999987</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -6503,7 +6503,7 @@
       </c>
       <c r="B2" s="60">
         <f>heat_demand_by_country_TWh!B2/heat_demand_by_country_TWh!$C$33</f>
-        <v>31.775626841666664</v>
+        <v>24.117432624999996</v>
       </c>
     </row>
     <row r="3" spans="1:42" s="50" customFormat="1">
@@ -6512,7 +6512,7 @@
       </c>
       <c r="B3" s="60">
         <f>heat_demand_by_country_TWh!B3/heat_demand_by_country_TWh!$C$33</f>
-        <v>48.929079466666657</v>
+        <v>37.543894099999996</v>
       </c>
     </row>
     <row r="4" spans="1:42" s="54" customFormat="1">
@@ -6521,7 +6521,7 @@
       </c>
       <c r="B4" s="62">
         <f>heat_demand_by_country_TWh!B4/heat_demand_by_country_TWh!$D$33</f>
-        <v>21.647185416666662</v>
+        <v>16.968614481481477</v>
       </c>
     </row>
     <row r="5" spans="1:42" s="54" customFormat="1">
@@ -6530,7 +6530,7 @@
       </c>
       <c r="B5" s="62">
         <f>heat_demand_by_country_TWh!B5/heat_demand_by_country_TWh!$D$33</f>
-        <v>10.986528694444441</v>
+        <v>8.8185744814814822</v>
       </c>
     </row>
     <row r="6" spans="1:42">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="B6" s="35">
         <f>heat_demand_by_country_TWh!B6/heat_demand_by_country_TWh!$B$33</f>
-        <v>4.6303778484848479</v>
+        <v>3.7110509015151516</v>
       </c>
     </row>
     <row r="7" spans="1:42" s="54" customFormat="1">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="B7" s="62">
         <f>heat_demand_by_country_TWh!B7/heat_demand_by_country_TWh!$D$33</f>
-        <v>34.090865768518526</v>
+        <v>20.101530777777775</v>
       </c>
     </row>
     <row r="8" spans="1:42" s="58" customFormat="1">
@@ -6557,7 +6557,7 @@
       </c>
       <c r="B8" s="61">
         <f>heat_demand_by_country_TWh!B8/heat_demand_by_country_TWh!$E$33</f>
-        <v>26.226079399999996</v>
+        <v>19.016925320000006</v>
       </c>
     </row>
     <row r="9" spans="1:42" s="58" customFormat="1">
@@ -6566,7 +6566,7 @@
       </c>
       <c r="B9" s="61">
         <f>heat_demand_by_country_TWh!B9/heat_demand_by_country_TWh!$E$33</f>
-        <v>2.5110753299999997</v>
+        <v>1.6376474399999998</v>
       </c>
     </row>
     <row r="10" spans="1:42" s="58" customFormat="1">
@@ -6575,7 +6575,7 @@
       </c>
       <c r="B10" s="61">
         <f>heat_demand_by_country_TWh!B10/heat_demand_by_country_TWh!$E$33</f>
-        <v>28.773557170000004</v>
+        <v>22.731954909999992</v>
       </c>
     </row>
     <row r="11" spans="1:42" s="50" customFormat="1">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="B11" s="60">
         <f>heat_demand_by_country_TWh!B11/heat_demand_by_country_TWh!$C$33</f>
-        <v>186.05819861666666</v>
+        <v>134.30679139166668</v>
       </c>
     </row>
     <row r="12" spans="1:42" s="50" customFormat="1">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="B12" s="60">
         <f>heat_demand_by_country_TWh!B12/heat_demand_by_country_TWh!$C$33</f>
-        <v>347.49039059166665</v>
+        <v>190.82753823333329</v>
       </c>
     </row>
     <row r="13" spans="1:42" s="46" customFormat="1">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="B13" s="59">
         <f>heat_demand_by_country_TWh!B13/heat_demand_by_country_TWh!$B$33</f>
-        <v>27.926583469696972</v>
+        <v>23.673801378787878</v>
       </c>
     </row>
     <row r="14" spans="1:42" s="46" customFormat="1">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="B14" s="59">
         <f>heat_demand_by_country_TWh!B14/heat_demand_by_country_TWh!$B$33</f>
-        <v>17.534884136363637</v>
+        <v>12.982014068181821</v>
       </c>
     </row>
     <row r="15" spans="1:42" s="50" customFormat="1">
@@ -6620,7 +6620,7 @@
       </c>
       <c r="B15" s="60">
         <f>heat_demand_by_country_TWh!B15/heat_demand_by_country_TWh!$C$33</f>
-        <v>11.130487741666665</v>
+        <v>9.4176021166666661</v>
       </c>
     </row>
     <row r="16" spans="1:42" s="46" customFormat="1">
@@ -6629,7 +6629,7 @@
       </c>
       <c r="B16" s="59">
         <f>heat_demand_by_country_TWh!B16/heat_demand_by_country_TWh!$B$33</f>
-        <v>156.66231618181817</v>
+        <v>131.83359767424238</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="58" customFormat="1">
@@ -6638,7 +6638,7 @@
       </c>
       <c r="B17" s="61">
         <f>heat_demand_by_country_TWh!B17/heat_demand_by_country_TWh!$E$33</f>
-        <v>4.4110236699999996</v>
+        <v>3.4997695000000002</v>
       </c>
     </row>
     <row r="18" spans="1:2" s="58" customFormat="1">
@@ -6647,7 +6647,7 @@
       </c>
       <c r="B18" s="61">
         <f>heat_demand_by_country_TWh!B18/heat_demand_by_country_TWh!$E$33</f>
-        <v>9.5964049100000004</v>
+        <v>7.043559909999999</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="50" customFormat="1">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="B19" s="60">
         <f>heat_demand_by_country_TWh!B19/heat_demand_by_country_TWh!$C$33</f>
-        <v>1.7964032166666666</v>
+        <v>1.3530466416666667</v>
       </c>
     </row>
     <row r="20" spans="1:2">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="B20" s="35">
         <f>heat_demand_by_country_TWh!B20/heat_demand_by_country_TWh!$B$33</f>
-        <v>1.2009696590909089</v>
+        <v>1.0364505681818181</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="50" customFormat="1">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="B21" s="60">
         <f>heat_demand_by_country_TWh!B21/heat_demand_by_country_TWh!$C$33</f>
-        <v>54.124373924999986</v>
+        <v>33.838843191666662</v>
       </c>
     </row>
     <row r="22" spans="1:2" s="54" customFormat="1">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="B22" s="62">
         <f>heat_demand_by_country_TWh!B22/heat_demand_by_country_TWh!$D$33</f>
-        <v>74.319034527777774</v>
+        <v>50.098428648148122</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="46" customFormat="1">
@@ -6692,7 +6692,7 @@
       </c>
       <c r="B23" s="59">
         <f>heat_demand_by_country_TWh!B23/heat_demand_by_country_TWh!$B$33</f>
-        <v>31.215002431818185</v>
+        <v>24.00222236363636</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="54" customFormat="1">
@@ -6701,7 +6701,7 @@
       </c>
       <c r="B24" s="62">
         <f>heat_demand_by_country_TWh!B24/heat_demand_by_country_TWh!$D$33</f>
-        <v>24.624637018518506</v>
+        <v>20.692283990740737</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="54" customFormat="1">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="B25" s="62">
         <f>heat_demand_by_country_TWh!B25/heat_demand_by_country_TWh!$D$33</f>
-        <v>11.106700851851851</v>
+        <v>8.8340030833333305</v>
       </c>
     </row>
     <row r="26" spans="1:2" s="46" customFormat="1">
@@ -6719,7 +6719,7 @@
       </c>
       <c r="B26" s="59">
         <f>heat_demand_by_country_TWh!B26/heat_demand_by_country_TWh!$B$33</f>
-        <v>3.7672030606060605</v>
+        <v>2.736857727272727</v>
       </c>
     </row>
     <row r="27" spans="1:2" s="46" customFormat="1">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="B27" s="59">
         <f>heat_demand_by_country_TWh!B27/heat_demand_by_country_TWh!$B$33</f>
-        <v>234.41479848484846</v>
+        <v>144.90774039393941</v>
       </c>
     </row>
     <row r="28" spans="1:2" s="58" customFormat="1">
@@ -6737,7 +6737,7 @@
       </c>
       <c r="B28" s="61">
         <f>heat_demand_by_country_TWh!B28/heat_demand_by_country_TWh!$E$33</f>
-        <v>36.815465860000003</v>
+        <v>25.972880719999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>